<commit_message>
update main.py with last changes
</commit_message>
<xml_diff>
--- a/app/users.xlsx
+++ b/app/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\funProject\chatbot\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B472691-5422-4A4E-B772-AFE48243D497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4474D0B-D3D6-4767-A128-73D77E4BC0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{44F5EEFC-D0C3-4298-AC8A-A4C380CADFD1}"/>
   </bookViews>
@@ -40,10 +40,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Shelton Teles</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Ellen Santilal</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -61,6 +57,10 @@
   </si>
   <si>
     <t>Ellen Youndiss Moisés Santilal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shelton</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -445,35 +445,35 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>20240175</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>20251266</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes in tge README
</commit_message>
<xml_diff>
--- a/app/users.xlsx
+++ b/app/users.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\funProject\chatbot\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4474D0B-D3D6-4767-A128-73D77E4BC0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4C58BF5-63F5-4D31-9DF6-27C04513BBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{44F5EEFC-D0C3-4298-AC8A-A4C380CADFD1}"/>
   </bookViews>
@@ -40,10 +40,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Ellen Santilal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>user_code</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -61,6 +57,10 @@
   </si>
   <si>
     <t>shelton</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ellen</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -445,35 +445,35 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>20240175</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>20251266</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>